<commit_message>
LØM-app 2.6.6: forkortelser forklart i appens innhold, rettet IB/UB
</commit_message>
<xml_diff>
--- a/pensum/ok02/OK02_Klasseoppgaver_v5.xlsx
+++ b/pensum/ok02/OK02_Klasseoppgaver_v5.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="158">
   <si>
-    <t xml:space="preserve">Klasseoppgaver til Økonomistyring kapittel 2: Viktige bedriftsøkonomiske begreper (V5)</t>
+    <t xml:space="preserve">Klasseoppgaver til Økonomistyring kapittel 2: Viktige bedriftsøkonomiske begreper (versjon 5)</t>
   </si>
   <si>
     <t xml:space="preserve">LØM · Fagskolen Oslo, Avdeling Elkraft · versjon 5, oktober 2026</t>
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Mai</t>
   </si>
   <si>
-    <t xml:space="preserve">Lager ved starten (IB)</t>
+    <t xml:space="preserve">Inngående lager (lageret ved starten)</t>
   </si>
   <si>
     <t xml:space="preserve">+ Varekjøp (utgift)</t>
   </si>
   <si>
-    <t xml:space="preserve">− Lager ved slutten (UB)</t>
+    <t xml:space="preserve">− Utgående lager (lageret ved slutten)</t>
   </si>
   <si>
     <t xml:space="preserve">= Varekostnad</t>
@@ -1224,7 +1224,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
         <v>28</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>520000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>

</xml_diff>